<commit_message>
Keep master-table photos inside their rows.
Shrink displayed part pictures so order numbers stay readable, and save the extra order added in the workbook.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data/part_machining_orders.xlsx
+++ b/data/part_machining_orders.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Orders" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Orders'!$A$1:$AA$25</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Orders'!$A$1:$AA$26</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -818,6 +818,31 @@
     </pic>
     <clientData/>
   </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>25</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="609600" cy="400050"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="25" name="Image 25" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId25"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
 </wsDr>
 </file>
 
@@ -1110,7 +1135,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AA25"/>
+  <dimension ref="A1:AA26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4107,8 +4132,119 @@
         <v>150</v>
       </c>
     </row>
+    <row r="26" ht="36" customHeight="1">
+      <c r="A26" s="12" t="inlineStr">
+        <is>
+          <t>APM-26065</t>
+        </is>
+      </c>
+      <c r="B26" s="13" t="n">
+        <v>46301</v>
+      </c>
+      <c r="C26" s="12" t="inlineStr">
+        <is>
+          <t>PO-45033</t>
+        </is>
+      </c>
+      <c r="D26" s="12" t="inlineStr">
+        <is>
+          <t>PN-2210</t>
+        </is>
+      </c>
+      <c r="E26" s="12" t="inlineStr">
+        <is>
+          <t>assets/parts/pn-2210.png</t>
+        </is>
+      </c>
+      <c r="F26" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="G26" s="13" t="n">
+        <v>46309</v>
+      </c>
+      <c r="H26" s="15" t="inlineStr">
+        <is>
+          <t>PCD 70 mm, 4 × Ø6.6 through, face Ra 1.6</t>
+        </is>
+      </c>
+      <c r="I26" s="12" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J26" s="12" t="inlineStr">
+        <is>
+          <t>Ø90 × 22 mm blank</t>
+        </is>
+      </c>
+      <c r="K26" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="L26" s="15" t="inlineStr">
+        <is>
+          <t>Ordered 02 Sep 2026</t>
+        </is>
+      </c>
+      <c r="M26" s="15" t="inlineStr">
+        <is>
+          <t>abc</t>
+        </is>
+      </c>
+      <c r="N26" s="15" t="inlineStr">
+        <is>
+          <t>afg</t>
+        </is>
+      </c>
+      <c r="O26" s="15" t="inlineStr">
+        <is>
+          <t>bbc</t>
+        </is>
+      </c>
+      <c r="P26" s="12" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="Q26" s="15" t="inlineStr"/>
+      <c r="R26" s="12" t="inlineStr">
+        <is>
+          <t>Incomplete</t>
+        </is>
+      </c>
+      <c r="S26" s="12" t="inlineStr">
+        <is>
+          <t>In-house</t>
+        </is>
+      </c>
+      <c r="T26" s="15" t="inlineStr"/>
+      <c r="U26" s="15" t="inlineStr"/>
+      <c r="V26" s="15" t="inlineStr"/>
+      <c r="W26" s="12" t="inlineStr">
+        <is>
+          <t>Astra</t>
+        </is>
+      </c>
+      <c r="X26" s="12" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="Y26" s="12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Z26" s="12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AA26" s="16" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AA25"/>
+  <autoFilter ref="A1:AA26"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>

</xml_diff>